<commit_message>
Refactor Excel model: Add Control & Checks sheets, dynamic peer comps, and scenario analysis
- Centralized hardcoded assumptions into a new Control sheet (growth, tax, WACC inputs)
- Built automated Checks sheet for model integrity (fixed Raw Data date bug in D13)
- Made historical column references dynamic
- Overhauled peer comps to be sector-aware and dynamic
- Fixed DCF growth logic (g = reinvestment x ROIC) and added 'REVIEW' verdict guard
- Added Bear/Base/Bull scenario selector and sensitivity grid
- Improved equity bridge (minority interest, leases)
</commit_message>
<xml_diff>
--- a/Consolidated Master Workbook For Dashboard.xlsx
+++ b/Consolidated Master Workbook For Dashboard.xlsx
@@ -1,166 +1,113 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\Advance Financial Project\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39A4B86F-925B-4B2F-A955-CF965DF5264C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{260A7F90-94FD-4B52-8C2C-301FFF211DCA}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId2"/>
-    <externalReference r:id="rId3"/>
-    <externalReference r:id="rId4"/>
-    <externalReference r:id="rId5"/>
-    <externalReference r:id="rId6"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
   </externalReferences>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
-  <si>
-    <t>Company</t>
-  </si>
-  <si>
-    <t>Current Market Price (₹)</t>
-  </si>
-  <si>
-    <t>DCF Intrinsic Value (₹)</t>
-  </si>
-  <si>
-    <t>Implied Price (EV/EBITDA)</t>
-  </si>
-  <si>
-    <t>Implied Price (P/E)</t>
-  </si>
-  <si>
-    <t>WACC (%)</t>
-  </si>
-  <si>
-    <t>Hind. Unilever</t>
-  </si>
-  <si>
-    <t>ITC</t>
-  </si>
-  <si>
-    <t>Nestle India</t>
-  </si>
-  <si>
-    <t>Varun Beverages</t>
-  </si>
-  <si>
-    <t>Britannia Inds.</t>
-  </si>
-  <si>
-    <t>PV of Explicit FCFF</t>
-  </si>
-  <si>
-    <t>PV of Terminal Value</t>
-  </si>
-  <si>
-    <t>Enterprise Value</t>
-  </si>
-  <si>
-    <t>Cash</t>
-  </si>
-  <si>
-    <t>Debt</t>
-  </si>
-  <si>
-    <t>Equity Value</t>
-  </si>
-  <si>
-    <t>Share Outstanding</t>
-  </si>
-  <si>
-    <t>Upside (%)</t>
-  </si>
-  <si>
-    <t>Valuation Recommendation</t>
-  </si>
-  <si>
-    <t>Return on Assets (%)</t>
-  </si>
-  <si>
-    <t>Return on Equity (%)</t>
-  </si>
-  <si>
-    <t>Altman's Score</t>
-  </si>
-  <si>
-    <t>EBITDA</t>
-  </si>
-  <si>
-    <t>Net Profit</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00;\(&quot;₹&quot;\ #,##0.0\);\-"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="+0.0%;-0.0%;0.0%"/>
+    <numFmt numFmtId="168" formatCode="+0.00%;-0.00%;0.00%"/>
+    <numFmt numFmtId="169" formatCode="&quot;₹&quot;\ #,##0.00;\(&quot;₹&quot;\ #,##0.00\);\-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="0"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00002060"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -171,8 +118,38 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+        <bgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+        <bgColor rgb="001F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -191,46 +168,185 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="00375623"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00375623"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="45">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="9" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="9" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Per cent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Profit &amp; Loss"/>
       <sheetName val="Quarters"/>
@@ -373,11 +489,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Profit &amp; Loss"/>
       <sheetName val="Quarters"/>
@@ -520,11 +633,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Profit &amp; Loss"/>
       <sheetName val="Quarters"/>
@@ -667,11 +777,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Profit &amp; Loss"/>
       <sheetName val="Quarters"/>
@@ -814,11 +921,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Profit &amp; Loss"/>
       <sheetName val="Quarters"/>
@@ -1276,499 +1380,1533 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A49D8CA5-98D0-49B3-992D-BA3144F59EB6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:U8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="1.88671875" customWidth="1"/>
-    <col min="2" max="2" width="21.77734375" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.88671875" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
-    <col min="7" max="7" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col width="1.88671875" customWidth="1" min="1" max="1"/>
+    <col width="21.77734375" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18.88671875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="18.88671875" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22.21875" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="15.88671875" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="16" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="18.21875" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="14.44140625" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="9.44140625" bestFit="1" customWidth="1" min="13" max="14"/>
+    <col width="11.88671875" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="15.88671875" bestFit="1" customWidth="1" min="16" max="16"/>
+    <col width="18.44140625" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="18.5546875" bestFit="1" customWidth="1" min="18" max="18"/>
+    <col width="13.6640625" bestFit="1" customWidth="1" min="19" max="19"/>
+    <col width="10.44140625" bestFit="1" customWidth="1" min="20" max="21"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="2:21" ht="5.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B4" s="2" t="s">
-        <v>6</v>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Current Market Price (₹)</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>DCF Intrinsic Value (₹)</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Upside (%)</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Valuation Recommendation</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Implied Price (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Implied Price (P/E)</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>WACC (%)</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>PV of Explicit FCFF</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>PV of Terminal Value</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>Enterprise Value</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>Debt</t>
+        </is>
+      </c>
+      <c r="O2" s="1" t="inlineStr">
+        <is>
+          <t>Equity Value</t>
+        </is>
+      </c>
+      <c r="P2" s="1" t="inlineStr">
+        <is>
+          <t>Share Outstanding</t>
+        </is>
+      </c>
+      <c r="Q2" s="1" t="inlineStr">
+        <is>
+          <t>Return on Assets (%)</t>
+        </is>
+      </c>
+      <c r="R2" s="1" t="inlineStr">
+        <is>
+          <t>Return on Equity (%)</t>
+        </is>
+      </c>
+      <c r="S2" s="1" t="inlineStr">
+        <is>
+          <t>Altman's Score</t>
+        </is>
+      </c>
+      <c r="T2" s="1" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="U2" s="1" t="inlineStr">
+        <is>
+          <t>Net Profit</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="5.4" customHeight="1"/>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Hind. Unilever</t>
+        </is>
       </c>
       <c r="C4" s="6">
         <f>[1]DCF!$D$43</f>
-        <v>2086.6</v>
+        <v/>
       </c>
       <c r="D4" s="6">
         <f>[1]DCF!$D$41</f>
-        <v>694.03283142872851</v>
+        <v/>
       </c>
       <c r="E4" s="4">
         <f>(D4-C4)/C4</f>
-        <v>-0.66738578001115278</v>
-      </c>
-      <c r="F4" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F4" s="5">
         <f>IF(E4 &gt; 0.1, "BUY", IF(E4 &lt; -0.1, "SELL", "HOLD"))</f>
-        <v>SELL</v>
+        <v/>
       </c>
       <c r="G4" s="6">
         <f>[1]Comp_Valuation!$P$36</f>
-        <v>2225.8699785656672</v>
+        <v/>
       </c>
       <c r="H4" s="6">
         <f>[1]Comp_Valuation!$Q$36</f>
-        <v>3264.2337243439592</v>
+        <v/>
       </c>
       <c r="I4" s="3">
         <f>[1]WACC!$K$46</f>
-        <v>0.11639541282808112</v>
+        <v/>
       </c>
       <c r="J4" s="6">
         <f>[1]DCF!$D$32</f>
-        <v>55644.395106485172</v>
+        <v/>
       </c>
       <c r="K4" s="6">
         <f>[1]DCF!$D$33</f>
-        <v>105654.95252012076</v>
+        <v/>
       </c>
       <c r="L4" s="6">
         <f>[1]DCF!$D$34</f>
-        <v>161299.34762660594</v>
+        <v/>
       </c>
       <c r="M4" s="6">
         <f>[1]DCF!$D$36</f>
-        <v>3248</v>
+        <v/>
       </c>
       <c r="N4" s="6">
         <f>[1]DCF!$D$37</f>
-        <v>1478</v>
+        <v/>
       </c>
       <c r="O4" s="6">
         <f>[1]DCF!$D$39</f>
-        <v>163069.34762660594</v>
+        <v/>
       </c>
       <c r="P4" s="7">
         <f>[1]DCF!$D$40</f>
-        <v>234.95912619999999</v>
+        <v/>
       </c>
       <c r="Q4" s="4">
         <f>'[1]Dupont Analysis'!$I$87</f>
-        <v>0.1884699970551563</v>
+        <v/>
       </c>
       <c r="R4" s="4">
         <f>'[1]Dupont Analysis'!$I$81</f>
-        <v>0.30649779399027932</v>
+        <v/>
       </c>
       <c r="S4" s="6">
         <f>'[1]Altman''s Z Score'!$I$93</f>
-        <v>11.590269955209473</v>
+        <v/>
       </c>
       <c r="T4" s="6">
         <f>'[1]Historical FS'!$L$19</f>
-        <v>18090</v>
+        <v/>
       </c>
       <c r="U4" s="6">
         <f>'[1]Historical FS'!$L$37</f>
-        <v>13187</v>
-      </c>
-    </row>
-    <row r="5" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B5" s="2" t="s">
-        <v>7</v>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
       </c>
       <c r="C5" s="6">
         <f>[2]DCF!$D$44</f>
-        <v>276.5</v>
+        <v/>
       </c>
       <c r="D5" s="6">
         <f>[2]DCF!$D$42</f>
-        <v>176.75907431058977</v>
+        <v/>
       </c>
       <c r="E5" s="4">
-        <f t="shared" ref="E5:E8" si="0">(D5-C5)/C5</f>
-        <v>-0.36072667518774043</v>
-      </c>
-      <c r="F5" s="5" t="str">
-        <f t="shared" ref="F5:F8" si="1">IF(E5 &gt; 0.1, "BUY", IF(E5 &lt; -0.1, "SELL", "HOLD"))</f>
-        <v>SELL</v>
+        <f>(D5-C5)/C5</f>
+        <v/>
+      </c>
+      <c r="F5" s="5">
+        <f>IF(E5 &gt; 0.1, "BUY", IF(E5 &lt; -0.1, "SELL", "HOLD"))</f>
+        <v/>
       </c>
       <c r="G5" s="6">
         <f>[2]Comp_Valuation!$P$37</f>
-        <v>782.08362718185617</v>
+        <v/>
       </c>
       <c r="H5" s="6">
         <f>[2]Comp_Valuation!$Q$37</f>
-        <v>852.35771829941496</v>
+        <v/>
       </c>
       <c r="I5" s="3">
         <f>[2]WACC!$K$46</f>
-        <v>0.11523601358805299</v>
+        <v/>
       </c>
       <c r="J5" s="6">
         <f>[2]DCF!$D$33</f>
-        <v>70746.76120442363</v>
+        <v/>
       </c>
       <c r="K5" s="6">
         <f>[2]DCF!$D$34</f>
-        <v>150113.22940712664</v>
+        <v/>
       </c>
       <c r="L5" s="6">
         <f>[2]DCF!$D$35</f>
-        <v>220859.99061155028</v>
+        <v/>
       </c>
       <c r="M5" s="6">
         <f>[2]DCF!$D$37</f>
-        <v>3008.79</v>
+        <v/>
       </c>
       <c r="N5" s="6">
         <f>[2]DCF!$D$38</f>
-        <v>2399.06</v>
+        <v/>
       </c>
       <c r="O5" s="6">
         <f>[2]DCF!$D$39</f>
-        <v>221469.72061155029</v>
+        <v/>
       </c>
       <c r="P5" s="7">
         <f>[2]DCF!$D$40</f>
-        <v>1252.9468231000001</v>
+        <v/>
       </c>
       <c r="Q5" s="4">
         <f>'[2]Dupont Analysis'!$I$96</f>
-        <v>0.2278075466899068</v>
+        <v/>
       </c>
       <c r="R5" s="4">
         <f>'[2]Dupont Analysis'!$I$78</f>
-        <v>0.29030243651927023</v>
+        <v/>
       </c>
       <c r="S5" s="6">
         <f>'[2]Altman''s Z Score'!$I$89</f>
-        <v>13.297686898728788</v>
+        <v/>
       </c>
       <c r="T5" s="6">
         <f>'[2]Historical FS'!$L$19</f>
-        <v>29630.879999999994</v>
+        <v/>
       </c>
       <c r="U5" s="6">
         <f>'[2]Historical FS'!$L$37</f>
-        <v>20819.939999999995</v>
-      </c>
-    </row>
-    <row r="6" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
-        <v>8</v>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Nestle India</t>
+        </is>
       </c>
       <c r="C6" s="6">
         <f>[3]DCF!$D$44</f>
-        <v>1498.8</v>
+        <v/>
       </c>
       <c r="D6" s="6">
         <f>[3]DCF!$D$42</f>
-        <v>1805.1432246522852</v>
+        <v/>
       </c>
       <c r="E6" s="4">
-        <f t="shared" si="0"/>
-        <v>0.20439233029909612</v>
-      </c>
-      <c r="F6" s="5" t="str">
-        <f t="shared" si="1"/>
-        <v>BUY</v>
+        <f>(D6-C6)/C6</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
+        <f>IF(E6 &gt; 0.1, "BUY", IF(E6 &lt; -0.1, "SELL", "HOLD"))</f>
+        <v/>
       </c>
       <c r="G6" s="6">
         <f>[3]Comp_Valuation!$P$37</f>
-        <v>915.06905057359052</v>
+        <v/>
       </c>
       <c r="H6" s="6">
         <f>[3]Comp_Valuation!$Q$37</f>
-        <v>932.34474679556968</v>
+        <v/>
       </c>
       <c r="I6" s="3">
         <f>[3]WACC!$K$46</f>
-        <v>0.11323696664251741</v>
+        <v/>
       </c>
       <c r="J6" s="6">
         <f>[3]DCF!$D$33</f>
-        <v>84650.940978145372</v>
+        <v/>
       </c>
       <c r="K6" s="6">
         <f>[3]DCF!$D$34</f>
-        <v>262540.70199665247</v>
+        <v/>
       </c>
       <c r="L6" s="6">
         <f>[3]DCF!$D$35</f>
-        <v>347191.64297479787</v>
+        <v/>
       </c>
       <c r="M6" s="6">
         <f>[3]DCF!$D$37</f>
-        <v>1340.87</v>
+        <v/>
       </c>
       <c r="N6" s="6">
         <f>[3]DCF!$D$38</f>
-        <v>444.16</v>
+        <v/>
       </c>
       <c r="O6" s="6">
         <f>[3]DCF!$D$39</f>
-        <v>348088.35297479789</v>
+        <v/>
       </c>
       <c r="P6" s="7">
         <f>[3]DCF!$D$40</f>
-        <v>192.83143200000001</v>
+        <v/>
       </c>
       <c r="Q6" s="4">
         <f>'[3]Dupont Analysis'!$I$96</f>
-        <v>0.27604779553491954</v>
+        <v/>
       </c>
       <c r="R6" s="4">
         <f>'[3]Dupont Analysis'!$I$78</f>
-        <v>0.75205884755457819</v>
+        <v/>
       </c>
       <c r="S6" s="6">
         <f>'[3]Altman''s Z Score'!$I$89</f>
-        <v>25.948427864655628</v>
+        <v/>
       </c>
       <c r="T6" s="6">
         <f>'[3]Historical FS'!$L$19</f>
-        <v>4746.0599999999995</v>
+        <v/>
       </c>
       <c r="U6" s="6">
         <f>'[3]Historical FS'!$L$37</f>
-        <v>2823.4699999999993</v>
-      </c>
-    </row>
-    <row r="7" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B7" s="2" t="s">
-        <v>9</v>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Varun Beverages</t>
+        </is>
       </c>
       <c r="C7" s="6">
         <f>[4]DCF!$D$44</f>
-        <v>436.25</v>
+        <v/>
       </c>
       <c r="D7" s="6">
         <f>[4]DCF!$D$42</f>
-        <v>92.11617570408221</v>
+        <v/>
       </c>
       <c r="E7" s="4">
-        <f t="shared" si="0"/>
-        <v>-0.78884544251213251</v>
-      </c>
-      <c r="F7" s="5" t="str">
-        <f t="shared" si="1"/>
-        <v>SELL</v>
+        <f>(D7-C7)/C7</f>
+        <v/>
+      </c>
+      <c r="F7" s="5">
+        <f>IF(E7 &gt; 0.1, "BUY", IF(E7 &lt; -0.1, "SELL", "HOLD"))</f>
+        <v/>
       </c>
       <c r="G7" s="6">
         <f>[4]Comp_Valuation!$P$37</f>
-        <v>588.4059373626759</v>
+        <v/>
       </c>
       <c r="H7" s="6">
         <f>[4]Comp_Valuation!$Q$37</f>
-        <v>504.1832295123391</v>
+        <v/>
       </c>
       <c r="I7" s="3">
         <f>[4]WACC!$K$46</f>
-        <v>0.11329045758465377</v>
+        <v/>
       </c>
       <c r="J7" s="6">
         <f>[4]DCF!$D$33</f>
-        <v>873.4899646644426</v>
+        <v/>
       </c>
       <c r="K7" s="6">
         <f>[4]DCF!$D$34</f>
-        <v>30789.787202779233</v>
+        <v/>
       </c>
       <c r="L7" s="6">
         <f>[4]DCF!$D$35</f>
-        <v>31663.277167443674</v>
+        <v/>
       </c>
       <c r="M7" s="6">
         <f>[4]DCF!$D$37</f>
-        <v>1998.49</v>
+        <v/>
       </c>
       <c r="N7" s="6">
         <f>[4]DCF!$D$38</f>
-        <v>2508.1799999999998</v>
+        <v/>
       </c>
       <c r="O7" s="6">
         <f>[4]DCF!$D$39</f>
-        <v>31153.587167443671</v>
+        <v/>
       </c>
       <c r="P7" s="7">
         <f>[4]DCF!$D$40</f>
-        <v>338.19887690000002</v>
+        <v/>
       </c>
       <c r="Q7" s="4">
         <f>'[4]Dupont Analysis'!$I$95</f>
-        <v>0.1247915083136734</v>
+        <v/>
       </c>
       <c r="R7" s="4">
         <f>'[4]Dupont Analysis'!$I$77</f>
-        <v>0.16781505079095502</v>
+        <v/>
       </c>
       <c r="S7" s="6">
         <f>'[4]Altman''s Z Score'!$I$88</f>
-        <v>19.330286392258877</v>
+        <v/>
       </c>
       <c r="T7" s="6">
         <f>'[4]Historical FS'!$L$19</f>
-        <v>5212.5399999999981</v>
+        <v/>
       </c>
       <c r="U7" s="6">
         <f>'[4]Historical FS'!$L$37</f>
-        <v>2852.489999999998</v>
-      </c>
-    </row>
-    <row r="8" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
-        <v>10</v>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Britannia Inds.</t>
+        </is>
       </c>
       <c r="C8" s="6">
         <f>[5]DCF!$D$44</f>
-        <v>5618</v>
+        <v/>
       </c>
       <c r="D8" s="6">
         <f>[5]DCF!$D$42</f>
-        <v>1007.3308700363914</v>
+        <v/>
       </c>
       <c r="E8" s="4">
-        <f t="shared" si="0"/>
-        <v>-0.82069582235023297</v>
-      </c>
-      <c r="F8" s="5" t="str">
-        <f t="shared" si="1"/>
-        <v>SELL</v>
+        <f>(D8-C8)/C8</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>IF(E8 &gt; 0.1, "BUY", IF(E8 &lt; -0.1, "SELL", "HOLD"))</f>
+        <v/>
       </c>
       <c r="G8" s="6">
         <f>[5]Comp_Valuation!$P$37</f>
-        <v>5009.9070639126694</v>
+        <v/>
       </c>
       <c r="H8" s="6">
         <f>[5]Comp_Valuation!$Q$37</f>
-        <v>5317.9952084867127</v>
+        <v/>
       </c>
       <c r="I8" s="3">
         <f>[5]WACC!$K$46</f>
-        <v>0.11330189423822679</v>
+        <v/>
       </c>
       <c r="J8" s="6">
         <f>[5]DCF!$D$33</f>
-        <v>2282.8442246806435</v>
+        <v/>
       </c>
       <c r="K8" s="6">
         <f>[5]DCF!$D$34</f>
-        <v>23008.402792705663</v>
+        <v/>
       </c>
       <c r="L8" s="6">
         <f>[5]DCF!$D$35</f>
-        <v>25291.247017386308</v>
+        <v/>
       </c>
       <c r="M8" s="6">
         <f>[5]DCF!$D$37</f>
-        <v>352.44</v>
+        <v/>
       </c>
       <c r="N8" s="6">
         <f>[5]DCF!$D$38</f>
-        <v>1380.28</v>
+        <v/>
       </c>
       <c r="O8" s="6">
         <f>[5]DCF!$D$39</f>
-        <v>24263.407017386307</v>
+        <v/>
       </c>
       <c r="P8" s="7">
         <f>[5]DCF!$D$40</f>
-        <v>24.086829600000002</v>
+        <v/>
       </c>
       <c r="Q8" s="4">
         <f>'[5]Dupont Analysis'!$I$95</f>
-        <v>0.27290143248234644</v>
+        <v/>
       </c>
       <c r="R8" s="4">
         <f>'[5]Dupont Analysis'!$I$77</f>
-        <v>0.53549250286400318</v>
+        <v/>
       </c>
       <c r="S8" s="6">
         <f>'[5]Altman''s Z Score'!$I$88</f>
-        <v>20.804261006663111</v>
+        <v/>
       </c>
       <c r="T8" s="6">
         <f>'[5]Historical FS'!$L$19</f>
-        <v>4356.130000000001</v>
+        <v/>
       </c>
       <c r="U8" s="6">
         <f>'[5]Historical FS'!$L$37</f>
-        <v>3154.7700000000009</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:M36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>INSTITUTIONAL MODEL CONTROL PANEL &amp; ASSUMPTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Single Source of Truth for Global Valuation Inputs, Scenarios &amp; Route Configuration</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>1. MODEL METADATA &amp; REPORTING SETTINGS</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n"/>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>COUNTRY</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>RISK-FREE (Rf)</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>ERP</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>MARGINAL TAX</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>SCENARIO</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>GROWTH MULT</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>MARGIN ADJ (NOT WIRED)</t>
+        </is>
+      </c>
+      <c r="M5" s="12" t="inlineStr">
+        <is>
+          <t>WACC SPREAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Valuation Date</t>
+        </is>
+      </c>
+      <c r="C6" s="14">
+        <f>TODAY()</f>
+        <v/>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>0.2517</v>
+      </c>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>1 - Bear Case</t>
+        </is>
+      </c>
+      <c r="K6" s="17" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L6" s="39" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="M6" s="40" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Reporting Currency</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>2 - Base Case</t>
+        </is>
+      </c>
+      <c r="K7" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Financial Reporting Unit</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Crores</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>3 - Bull Case</t>
+        </is>
+      </c>
+      <c r="K8" s="17" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L8" s="39" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M8" s="40" t="n">
+        <v>-0.005</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Unit Scale Factor</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Target Country</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>0.3062</v>
+      </c>
+      <c r="J10" s="22" t="inlineStr">
+        <is>
+          <t>ACTIVE MULTIPLIERS:</t>
+        </is>
+      </c>
+      <c r="K10" s="23">
+        <f>CHOOSE(C14, K6, K7, K8)</f>
+        <v/>
+      </c>
+      <c r="L10" s="41">
+        <f>CHOOSE(C14, L6, L7, L8)</f>
+        <v/>
+      </c>
+      <c r="M10" s="42">
+        <f>CHOOSE(C14, M6, M7, M8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Target Sector / Industry</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>Corporate / Non-Financial</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Valuation Framework Switch</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>FCFF DCF</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Benchmark Market Index</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>NIFTY 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Active Valuation Scenario</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>2. COST OF CAPITAL &amp; DCF ASSUMPTIONS</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Risk-Free Rate (Rf)</t>
+        </is>
+      </c>
+      <c r="C17" s="27">
+        <f>VLOOKUP(C10, E6:H12, 2, FALSE())</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Equity Risk Premium (ERP)</t>
+        </is>
+      </c>
+      <c r="C18" s="27">
+        <f>VLOOKUP(C10, E6:H12, 3, FALSE())</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Marginal Corporate Tax Rate</t>
+        </is>
+      </c>
+      <c r="C19" s="27">
+        <f>VLOOKUP(C10, E6:H12, 4, FALSE())</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Effective Dynamic Tax Rate</t>
+        </is>
+      </c>
+      <c r="C20" s="27">
+        <f>MEDIAN(MAX(0.15, MIN(0.35, INDEX('Data Sheet'!$B29:$K29, C26)/MAX(1, INDEX('Data Sheet'!$B28:$K28, C26)))), C19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Terminal Growth Rate (g)</t>
+        </is>
+      </c>
+      <c r="C21" s="27" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Reinvestment Rate Ceiling</t>
+        </is>
+      </c>
+      <c r="C22" s="27" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Investments Fair-Value Haircut</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Minority Interest Method</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>Book Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>3. DYNAMIC STATEMENT PERIOD SELECTOR</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Latest Historical Period Column Index</t>
+        </is>
+      </c>
+      <c r="C26" s="28">
+        <f>MATCH(MAX('Data Sheet'!$B56:$K56), 'Data Sheet'!$B56:$K56, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Latest Statement Header Date</t>
+        </is>
+      </c>
+      <c r="C27" s="29">
+        <f>INDEX('Data Sheet'!$B56:$K56, C26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Latest Stock Price (Data Sheet)</t>
+        </is>
+      </c>
+      <c r="C28" s="43">
+        <f>'Data Sheet'!B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Default Credit Spread over Rf (used when debt is negligible)</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="n">
+        <v>0.015</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Max Credit Spread Cap (calc outside Rf..Rf+cap is rejected)</t>
+        </is>
+      </c>
+      <c r="C30" s="27" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>4. OPTIONAL ALTERNATE 10-YEAR DCF (parallel view - base DCF unchanged)</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Year-1 EBIT Growth Override (blank = use model)</t>
+        </is>
+      </c>
+      <c r="C33" s="44" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Exit EV/EBIT Multiple (x)</t>
+        </is>
+      </c>
+      <c r="C34" s="26" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Terminal Method (Gordon Growth / Exit Multiple)</t>
+        </is>
+      </c>
+      <c r="C35" s="20" t="inlineStr">
+        <is>
+          <t>Gordon Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Incremental ROIC Override (blank = model ROIC)</t>
+        </is>
+      </c>
+      <c r="C36" s="44" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:F21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>MODEL AUDIT &amp; INTEGRITY CHECK PANEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="31" t="inlineStr">
+        <is>
+          <t>OVERALL MODEL STATUS:</t>
+        </is>
+      </c>
+      <c r="C3" s="32">
+        <f>IF(AND(F6="PASS", F7="PASS", F8="PASS", F9="PASS", F10="PASS", F11="PASS", F12="PASS", F13="PASS", F14="PASS", F15="PASS"), "MODEL STATUS: OK", "MODEL STATUS: CHECK REQUIRED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="33" t="inlineStr">
+        <is>
+          <t>CHECK ITEM</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>VALIDATION LOGIC &amp; FORMULA</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>CURRENT VALUE / VARIANCE</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>THRESHOLD</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>1. Balance Sheet Identity</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Total liabilities side ties to its components and to total assets</t>
+        </is>
+      </c>
+      <c r="D6" s="35">
+        <f>MAX(ABS(INDEX('Data Sheet'!$B61:$K61,Control!$C$26)-(INDEX('Data Sheet'!$B57:$K57,Control!$C$26)+INDEX('Data Sheet'!$B58:$K58,Control!$C$26)+INDEX('Data Sheet'!$B59:$K59,Control!$C$26)+INDEX('Data Sheet'!$B60:$K60,Control!$C$26))),ABS(INDEX('Data Sheet'!$B61:$K61,Control!$C$26)-INDEX('Data Sheet'!$B66:$K66,Control!$C$26)))</f>
+        <v/>
+      </c>
+      <c r="E6" s="36" t="inlineStr">
+        <is>
+          <t>&lt; ₹ 5.0 Cr</t>
+        </is>
+      </c>
+      <c r="F6" s="37">
+        <f>IF(D6&lt;5, "PASS", "CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="34" t="inlineStr">
+        <is>
+          <t>2. PBT Mathematical Tie</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Sales less all expenses plus other income less depreciation and interest ties to PBT</t>
+        </is>
+      </c>
+      <c r="D7" s="38">
+        <f>ABS(INDEX('Data Sheet'!$B17:$K17,Control!$C$26)-SUM(INDEX('Data Sheet'!$B$18:$K$24,0,Control!$C$26))+INDEX('Data Sheet'!$B25:$K25,Control!$C$26)-INDEX('Data Sheet'!$B26:$K26,Control!$C$26)-INDEX('Data Sheet'!$B27:$K27,Control!$C$26)-INDEX('Data Sheet'!$B28:$K28,Control!$C$26))/MAX(1,INDEX('Data Sheet'!$B28:$K28,Control!$C$26))</f>
+        <v/>
+      </c>
+      <c r="E7" s="36" t="inlineStr">
+        <is>
+          <t>&lt; 1.5%</t>
+        </is>
+      </c>
+      <c r="F7" s="37">
+        <f>IF(D7&lt;0.015, "PASS", "CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="34" t="inlineStr">
+        <is>
+          <t>3. Debt Schedule Concordance</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Data Sheet Borrowings ties to the independently pasted Raw FS borrowings (latest year)</t>
+        </is>
+      </c>
+      <c r="D8" s="35">
+        <f>ABS(INDEX('Data Sheet'!$B59:$K59,Control!$C$26)-LOOKUP(2,1/ISNUMBER('Raw FS'!$C7:$N7),'Raw FS'!$C7:$N7))</f>
+        <v/>
+      </c>
+      <c r="E8" s="36" t="inlineStr">
+        <is>
+          <t>&lt; ₹ 5.0 Cr</t>
+        </is>
+      </c>
+      <c r="F8" s="37">
+        <f>IF(D8&lt;5, "PASS", "CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="34" t="inlineStr">
+        <is>
+          <t>4. P&amp;L Expenses Agreement</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Data Sheet total expenses (rows 18-24) tie to Raw FS total expenses</t>
+        </is>
+      </c>
+      <c r="D9" s="35">
+        <f>ABS(SUM(INDEX('Data Sheet'!$B$18:$K$24,0,Control!$C$26))-'Raw FS'!AD5)</f>
+        <v/>
+      </c>
+      <c r="E9" s="36" t="inlineStr">
+        <is>
+          <t>&lt; ₹ 10.0 Cr</t>
+        </is>
+      </c>
+      <c r="F9" s="37">
+        <f>IF(D9&lt;10, "PASS", "CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="34" t="inlineStr">
+        <is>
+          <t>5. Formula Error Counter</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Zero formula errors on Summary, DCF, WACC, Intrinsic Valuation, Comps and Beta tabs</t>
+        </is>
+      </c>
+      <c r="D10" s="35">
+        <f>SUMPRODUCT(--ISERROR('AI Valuation Summary'!A4:H47))+SUMPRODUCT(--ISERROR(DCF!A1:M55))+SUMPRODUCT(--ISERROR(WACC!A1:K46))+SUMPRODUCT(--ISERROR('Intrinsic Valuation'!A1:L65))+SUMPRODUCT(--ISERROR(Comp_Valuation!A1:Q39))+SUMPRODUCT(--ISERROR('Beta-Regression'!A1:O302))</f>
+        <v/>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>0 Errors</t>
+        </is>
+      </c>
+      <c r="F10" s="37">
+        <f>IF(D10=0, "PASS", "CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t>6. Terminal Value EV Share</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>Terminal Value percentage of Enterprise Value is sustainable</t>
+        </is>
+      </c>
+      <c r="D11" s="38">
+        <f>DCF!D34 / MAX(1, DCF!D35)</f>
+        <v/>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>&lt; 75.0%</t>
+        </is>
+      </c>
+      <c r="F11" s="37">
+        <f>IF(D11&lt;0.75, "PASS", "CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="34" t="inlineStr">
+        <is>
+          <t>7. Growth vs WACC Boundary</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Terminal growth rate is less than WACC and within Risk-Free rate</t>
+        </is>
+      </c>
+      <c r="D12" s="38">
+        <f>DCF!D20 - DCF!D19</f>
+        <v/>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>&gt; 0.5%</t>
+        </is>
+      </c>
+      <c r="F12" s="37">
+        <f>IF(AND(D12&gt;0.005, DCF!D19&lt;=Control!$C$17), "PASS", "CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>8. Trading Price Freshness</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Market trading price quote is within acceptable institutional window</t>
+        </is>
+      </c>
+      <c r="D13" s="35">
+        <f>TODAY()-SUMPRODUCT(MAX(IFERROR(DATEVALUE('Raw Data'!G6:G252),IF(ISNUMBER('Raw Data'!G6:G252),'Raw Data'!G6:G252,0))))</f>
+        <v/>
+      </c>
+      <c r="E13" s="36" t="inlineStr">
+        <is>
+          <t>&lt;= 45 Days</t>
+        </is>
+      </c>
+      <c r="F13" s="37">
+        <f>IF(D13&lt;=45, "PASS", "CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="34" t="inlineStr">
+        <is>
+          <t>9. Peer Group Sample Size</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>Comparable peer valuation set contains minimum robust observations</t>
+        </is>
+      </c>
+      <c r="D14" s="35">
+        <f>COUNTA(Comp_Valuation!C12:C26)</f>
+        <v/>
+      </c>
+      <c r="E14" s="36" t="inlineStr">
+        <is>
+          <t>&gt;= 4 Peers</t>
+        </is>
+      </c>
+      <c r="F14" s="37">
+        <f>IF(D14&gt;=4, "PASS", "CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="34" t="inlineStr">
+        <is>
+          <t>10. DCF Bridge Mathematical Tie</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Equity Value equals EV + Cash + Investments - Debt - Minority Interest</t>
+        </is>
+      </c>
+      <c r="D15" s="35">
+        <f>ABS(DCF!D40 - (DCF!D35 + DCF!D37 - DCF!D38 - DCF!D39))</f>
+        <v/>
+      </c>
+      <c r="E15" s="36" t="inlineStr">
+        <is>
+          <t>&lt; ₹ 0.01</t>
+        </is>
+      </c>
+      <c r="F15" s="37">
+        <f>IF(D15&lt;0.01, "PASS", "CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>ADVISORY CHECKS (informational - NOT included in overall status)</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="34" t="inlineStr">
+        <is>
+          <t>A1. DCF vs Market Divergence</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Absolute gap between DCF value per share and market price</t>
+        </is>
+      </c>
+      <c r="D18" s="38">
+        <f>ABS(DCF!D46)</f>
+        <v/>
+      </c>
+      <c r="E18" s="36" t="inlineStr">
+        <is>
+          <t>&lt; 50%</t>
+        </is>
+      </c>
+      <c r="F18" s="37">
+        <f>IF(D18&lt;0.5,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="34" t="inlineStr">
+        <is>
+          <t>A2. WACC Sanity Range</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>WACC sits inside a plausible band for the target market</t>
+        </is>
+      </c>
+      <c r="D19" s="38">
+        <f>DCF!D20</f>
+        <v/>
+      </c>
+      <c r="E19" s="36" t="inlineStr">
+        <is>
+          <t>8% - 16%</t>
+        </is>
+      </c>
+      <c r="F19" s="37">
+        <f>IF(AND(D19&gt;=0.08,D19&lt;=0.16),"PASS","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="34" t="inlineStr">
+        <is>
+          <t>A3. Market Cap Tie</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>Market cap used in WACC weights ties to Price x Shares on Data Sheet</t>
+        </is>
+      </c>
+      <c r="D20" s="38">
+        <f>ABS(WACC!C35/'Data Sheet'!B9-1)</f>
+        <v/>
+      </c>
+      <c r="E20" s="36" t="inlineStr">
+        <is>
+          <t>&lt; 2%</t>
+        </is>
+      </c>
+      <c r="F20" s="37">
+        <f>IF(D20&lt;0.02,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t>A4. Reinvestment History Spike</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Largest historical reinvestment rate (blank-year / acquisition spikes distort median)</t>
+        </is>
+      </c>
+      <c r="D21" s="38">
+        <f>MAX('Intrinsic Valuation'!H52:L52)</f>
+        <v/>
+      </c>
+      <c r="E21" s="36" t="inlineStr">
+        <is>
+          <t>&lt;= 100%</t>
+        </is>
+      </c>
+      <c r="F21" s="37">
+        <f>IF(D21&lt;=1,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>